<commit_message>
Added code to add 2022 pw samples to updated inventory
</commit_message>
<xml_diff>
--- a/processing_scripts/Inventory_Processing/2022 Metadata Creation/T3 TMP Data Sheet.xlsx
+++ b/processing_scripts/Inventory_Processing/2022 Metadata Creation/T3 TMP Data Sheet.xlsx
@@ -51,12 +51,18 @@
     <t>15mL Falcon Tube</t>
   </si>
   <si>
+    <t>—</t>
+  </si>
+  <si>
     <t>2mL Glass Vial</t>
   </si>
   <si>
     <t>40mL Amber Vials</t>
   </si>
   <si>
+    <t>OO</t>
+  </si>
+  <si>
     <t>2mL Plastic Orange Cap Vial</t>
   </si>
   <si>
@@ -66,12 +72,6 @@
     <t xml:space="preserve">Prep for next sampling and Notes </t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>OO</t>
-  </si>
-  <si>
     <t>DOC (min 7ml; max 10)</t>
   </si>
   <si>
@@ -123,22 +123,25 @@
     <t>General note: raining relatively hard, but not pouring. Pools near many of the lysimeters but not as many or as large as during water treatment</t>
   </si>
   <si>
+    <t>C6</t>
+  </si>
+  <si>
     <t>General note: Vibes- wet AF aka drowned rat</t>
   </si>
   <si>
-    <t>C6</t>
-  </si>
-  <si>
     <t>Dead frog near lysimeter</t>
   </si>
   <si>
     <t>F4</t>
   </si>
   <si>
+    <t xml:space="preserve">CONTROL </t>
+  </si>
+  <si>
     <t>H3</t>
   </si>
   <si>
-    <t xml:space="preserve">CONTROL </t>
+    <t>less than 1, discarded</t>
   </si>
   <si>
     <t>H6</t>
@@ -147,7 +150,7 @@
     <t>B4</t>
   </si>
   <si>
-    <t>less than 1, discarded</t>
+    <t>got knocked or not sealed properly, no pressure built</t>
   </si>
   <si>
     <t>D5</t>
@@ -159,13 +162,10 @@
     <t>F6</t>
   </si>
   <si>
+    <t>lost a couple mLs of pooled samples</t>
+  </si>
+  <si>
     <t>I5</t>
-  </si>
-  <si>
-    <t>got knocked or not sealed properly, no pressure built</t>
-  </si>
-  <si>
-    <t>lost a couple mLs of pooled samples</t>
   </si>
   <si>
     <t>dry</t>
@@ -257,14 +257,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FF00DA63"/>
+        <bgColor rgb="FF00DA63"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00DA63"/>
-        <bgColor rgb="FF00DA63"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -365,12 +365,12 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="20" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="20" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
@@ -379,6 +379,9 @@
     </xf>
     <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
@@ -396,9 +399,6 @@
     <xf borderId="3" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
     <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -431,6 +431,9 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
+    <xf borderId="2" fillId="8" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -440,19 +443,16 @@
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -464,38 +464,38 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -825,13 +825,13 @@
       <c r="C3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>0.40347222222222223</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="6">
         <v>0.4861111111111111</v>
       </c>
       <c r="G3" s="2"/>
@@ -846,7 +846,7 @@
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="2"/>
@@ -883,33 +883,33 @@
       <c r="A6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="15" t="s">
+      <c r="D6" s="14"/>
+      <c r="E6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="13"/>
+      <c r="G6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="14"/>
       <c r="I6" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="J6" s="14"/>
       <c r="K6" s="19"/>
       <c r="L6" s="20" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="M6" s="21"/>
-      <c r="N6" s="13"/>
+      <c r="N6" s="14"/>
       <c r="O6" s="22"/>
     </row>
     <row r="7">
@@ -942,24 +942,24 @@
       <c r="K7" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="L7" s="30" t="s">
+      <c r="L7" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="M7" s="31" t="s">
+      <c r="M7" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="N7" s="30" t="s">
+      <c r="N7" s="31" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B8" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="36">
         <v>10.0</v>
       </c>
       <c r="D8" s="37">
@@ -977,11 +977,11 @@
       <c r="H8" s="37">
         <v>1.5</v>
       </c>
-      <c r="I8" s="35">
+      <c r="I8" s="36">
         <v>25.0</v>
       </c>
       <c r="J8" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K8" s="37"/>
       <c r="L8" s="37" t="s">
@@ -995,35 +995,35 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" s="39">
         <v>7.0</v>
       </c>
       <c r="D9" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E9" s="40">
         <v>1.5</v>
       </c>
       <c r="F9" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G9" s="40">
         <v>1.5</v>
       </c>
       <c r="H9" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I9" s="39">
         <v>0.5</v>
       </c>
       <c r="J9" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K9" s="40"/>
       <c r="L9" s="40" t="s">
@@ -1037,13 +1037,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="36">
         <v>7.0</v>
       </c>
       <c r="D10" s="37">
@@ -1053,22 +1053,22 @@
         <v>1.5</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H10" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" s="35">
+        <v>12</v>
+      </c>
+      <c r="I10" s="36">
         <v>1.0</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
       <c r="M10" s="37">
         <v>13.0</v>
       </c>
@@ -1077,38 +1077,38 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="39">
         <v>7.0</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E11" s="40">
         <v>1.5</v>
       </c>
       <c r="F11" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H11" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I11" s="39">
         <v>0.5</v>
       </c>
       <c r="J11" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K11" s="46"/>
+      <c r="L11" s="46"/>
       <c r="M11" s="40">
         <v>9.0</v>
       </c>
@@ -1117,13 +1117,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="35">
+        <v>43</v>
+      </c>
+      <c r="C12" s="36">
         <v>7.0</v>
       </c>
       <c r="D12" s="37">
@@ -1141,14 +1141,14 @@
       <c r="H12" s="37">
         <v>1.5</v>
       </c>
-      <c r="I12" s="35">
+      <c r="I12" s="36">
         <v>0.5</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K12" s="45"/>
+      <c r="L12" s="45"/>
       <c r="M12" s="37">
         <v>30.0</v>
       </c>
@@ -1157,38 +1157,38 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" s="39">
         <v>10.0</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E13" s="40">
         <v>1.5</v>
       </c>
       <c r="F13" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H13" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" s="47">
+        <v>12</v>
+      </c>
+      <c r="I13" s="51">
         <v>25.0</v>
       </c>
       <c r="J13" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K13" s="46"/>
+      <c r="L13" s="46"/>
       <c r="M13" s="40">
         <v>64.0</v>
       </c>
@@ -1197,38 +1197,38 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B14" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="35">
+        <v>46</v>
+      </c>
+      <c r="C14" s="36">
         <v>7.0</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E14" s="37">
         <v>1.5</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G14" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H14" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" s="35">
+        <v>12</v>
+      </c>
+      <c r="I14" s="36">
         <v>7.0</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K14" s="41"/>
-      <c r="L14" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K14" s="45"/>
+      <c r="L14" s="45"/>
       <c r="M14" s="37">
         <v>17.0</v>
       </c>
@@ -1237,38 +1237,38 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" s="39">
         <v>7.0</v>
       </c>
       <c r="D15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E15" s="40">
         <v>1.5</v>
       </c>
       <c r="F15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I15" s="39">
         <v>12.0</v>
       </c>
       <c r="J15" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K15" s="43"/>
-      <c r="L15" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K15" s="46"/>
+      <c r="L15" s="46"/>
       <c r="M15" s="40">
         <v>23.0</v>
       </c>
@@ -1277,38 +1277,38 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B16" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="35">
+        <v>48</v>
+      </c>
+      <c r="C16" s="36">
         <v>10.0</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E16" s="37">
         <v>1.5</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G16" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H16" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="35">
+        <v>12</v>
+      </c>
+      <c r="I16" s="36">
         <v>25.0</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K16" s="41"/>
-      <c r="L16" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K16" s="45"/>
+      <c r="L16" s="45"/>
       <c r="M16" s="37">
         <v>67.0</v>
       </c>
@@ -1317,38 +1317,38 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C17" s="39">
         <v>10.0</v>
       </c>
       <c r="D17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E17" s="40">
         <v>1.5</v>
       </c>
       <c r="F17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I17" s="39">
         <v>25.0</v>
       </c>
       <c r="J17" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K17" s="43"/>
-      <c r="L17" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K17" s="46"/>
+      <c r="L17" s="46"/>
       <c r="M17" s="40">
         <v>92.0</v>
       </c>
@@ -1449,13 +1449,13 @@
       <c r="C3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>4</v>
       </c>
       <c r="G3" s="2"/>
@@ -1505,33 +1505,33 @@
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="15" t="s">
+      <c r="D6" s="14"/>
+      <c r="E6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="13"/>
+      <c r="G6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="14"/>
       <c r="I6" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="J6" s="14"/>
       <c r="K6" s="19"/>
       <c r="L6" s="20" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="M6" s="21"/>
-      <c r="N6" s="13"/>
+      <c r="N6" s="14"/>
     </row>
     <row r="7">
       <c r="A7" s="23"/>
@@ -1563,24 +1563,24 @@
       <c r="K7" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="L7" s="30" t="s">
+      <c r="L7" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="M7" s="31" t="s">
+      <c r="M7" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="N7" s="30" t="s">
+      <c r="N7" s="31" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B8" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="36">
         <v>10.0</v>
       </c>
       <c r="D8" s="37">
@@ -1598,15 +1598,15 @@
       <c r="H8" s="37">
         <v>1.5</v>
       </c>
-      <c r="I8" s="35">
+      <c r="I8" s="36">
         <v>25.0</v>
       </c>
       <c r="J8" s="37" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K8" s="37"/>
       <c r="L8" s="37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M8" s="37">
         <f>60+30+60+23</f>
@@ -1617,11 +1617,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" s="39">
         <v>7.0</v>
@@ -1645,10 +1645,10 @@
         <v>0.0</v>
       </c>
       <c r="J9" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K9" s="43"/>
-      <c r="L9" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K9" s="46"/>
+      <c r="L9" s="46"/>
       <c r="M9" s="40">
         <v>32.0</v>
       </c>
@@ -1657,13 +1657,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B10" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="36">
         <v>7.0</v>
       </c>
       <c r="D10" s="37">
@@ -1681,14 +1681,14 @@
       <c r="H10" s="37">
         <v>1.5</v>
       </c>
-      <c r="I10" s="35">
+      <c r="I10" s="36">
         <v>4.0</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
       <c r="M10" s="37">
         <v>49.0</v>
       </c>
@@ -1697,11 +1697,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="39">
         <v>10.0</v>
@@ -1725,10 +1725,10 @@
         <v>0.0</v>
       </c>
       <c r="J11" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K11" s="46"/>
+      <c r="L11" s="46"/>
       <c r="M11" s="40">
         <f>56+45+53</f>
         <v>154</v>
@@ -1738,13 +1738,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="35">
+        <v>43</v>
+      </c>
+      <c r="C12" s="36">
         <v>10.0</v>
       </c>
       <c r="D12" s="37">
@@ -1762,14 +1762,14 @@
       <c r="H12" s="37">
         <v>1.5</v>
       </c>
-      <c r="I12" s="35">
+      <c r="I12" s="36">
         <v>25.0</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K12" s="45"/>
+      <c r="L12" s="45"/>
       <c r="M12" s="37">
         <f>60+57</f>
         <v>117</v>
@@ -1779,38 +1779,38 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" s="39">
         <v>7.0</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E13" s="37">
         <v>1.5</v>
       </c>
       <c r="F13" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H13" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I13" s="39">
         <v>9.0</v>
       </c>
       <c r="J13" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K13" s="46"/>
+      <c r="L13" s="46"/>
       <c r="M13" s="40">
         <v>18.0</v>
       </c>
@@ -1819,38 +1819,38 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B14" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="35">
+        <v>46</v>
+      </c>
+      <c r="C14" s="36">
         <v>10.0</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E14" s="37">
         <v>1.5</v>
       </c>
       <c r="F14" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G14" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H14" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" s="35">
+        <v>12</v>
+      </c>
+      <c r="I14" s="36">
         <v>25.0</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K14" s="41"/>
-      <c r="L14" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K14" s="45"/>
+      <c r="L14" s="45"/>
       <c r="M14" s="37">
         <f>62+60+59+3</f>
         <v>184</v>
@@ -1860,38 +1860,38 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" s="39">
         <v>7.0</v>
       </c>
       <c r="D15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E15" s="37">
         <v>1.5</v>
       </c>
       <c r="F15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H15" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I15" s="39">
         <v>19.0</v>
       </c>
       <c r="J15" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K15" s="43"/>
-      <c r="L15" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K15" s="46"/>
+      <c r="L15" s="46"/>
       <c r="M15" s="40">
         <v>28.0</v>
       </c>
@@ -1900,38 +1900,38 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B16" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="35">
+        <v>48</v>
+      </c>
+      <c r="C16" s="36">
         <v>7.0</v>
       </c>
       <c r="D16" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E16" s="37">
         <v>1.5</v>
       </c>
       <c r="F16" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G16" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H16" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="35">
+        <v>12</v>
+      </c>
+      <c r="I16" s="36">
         <v>6.0</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K16" s="41"/>
-      <c r="L16" s="41"/>
+        <v>12</v>
+      </c>
+      <c r="K16" s="45"/>
+      <c r="L16" s="45"/>
       <c r="M16" s="37">
         <v>15.0</v>
       </c>
@@ -1940,38 +1940,38 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="35" t="s">
         <v>33</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C17" s="39">
         <v>10.0</v>
       </c>
       <c r="D17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E17" s="37">
         <v>1.5</v>
       </c>
       <c r="F17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H17" s="40" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I17" s="39">
         <v>25.0</v>
       </c>
       <c r="J17" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K17" s="43"/>
-      <c r="L17" s="43"/>
+        <v>12</v>
+      </c>
+      <c r="K17" s="46"/>
+      <c r="L17" s="46"/>
       <c r="M17" s="40">
         <f>25+35+47</f>
         <v>107</v>
@@ -2072,20 +2072,20 @@
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="11">
         <v>44735.0</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>0.4013888888888889</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>17</v>
+      <c r="F3" s="7" t="s">
+        <v>12</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -2100,8 +2100,8 @@
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>18</v>
+      <c r="B4" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -2135,36 +2135,36 @@
       <c r="N5" s="3"/>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="15" t="s">
+      <c r="D6" s="14"/>
+      <c r="E6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="13"/>
+      <c r="G6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="14"/>
       <c r="I6" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="J6" s="14"/>
       <c r="K6" s="19"/>
       <c r="L6" s="20" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="M6" s="21"/>
-      <c r="N6" s="13"/>
+      <c r="N6" s="14"/>
     </row>
     <row r="7">
       <c r="A7" s="23"/>
@@ -2196,433 +2196,433 @@
       <c r="K7" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="L7" s="30" t="s">
+      <c r="L7" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="M7" s="42" t="s">
+      <c r="M7" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="N7" s="30" t="s">
+      <c r="N7" s="31" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="M8" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="N8" s="44">
+        <v>46.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="49">
+        <v>7.5</v>
+      </c>
+      <c r="D9" s="47">
+        <v>3.0</v>
+      </c>
+      <c r="E9" s="50">
+        <v>1.5</v>
+      </c>
+      <c r="F9" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="H9" s="47">
+        <v>1.5</v>
+      </c>
+      <c r="I9" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="K9" s="47"/>
+      <c r="L9" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="M9" s="47">
+        <v>20.0</v>
+      </c>
+      <c r="N9" s="47">
+        <v>49.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J10" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="M10" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="N10" s="50">
+        <v>49.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" s="46"/>
-      <c r="L8" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="M8" s="48" t="s">
+      <c r="C11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="M11" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="N11" s="47">
+        <v>47.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="44">
+        <v>7.5</v>
+      </c>
+      <c r="D12" s="50">
+        <v>3.5</v>
+      </c>
+      <c r="E12" s="50">
+        <v>1.5</v>
+      </c>
+      <c r="F12" s="50">
+        <v>30.0</v>
+      </c>
+      <c r="G12" s="50">
+        <v>1.5</v>
+      </c>
+      <c r="H12" s="50">
+        <v>1.5</v>
+      </c>
+      <c r="I12" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="K12" s="50"/>
+      <c r="L12" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="M12" s="50">
+        <v>45.0</v>
+      </c>
+      <c r="N12" s="50">
+        <v>46.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="N8" s="46">
+      <c r="C13" s="49">
+        <v>8.0</v>
+      </c>
+      <c r="D13" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="50">
+        <v>1.5</v>
+      </c>
+      <c r="F13" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" s="49">
+        <v>18.0</v>
+      </c>
+      <c r="J13" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="K13" s="47"/>
+      <c r="L13" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="M13" s="47">
+        <v>30.0</v>
+      </c>
+      <c r="N13" s="47">
+        <v>49.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="44">
+        <v>1.5</v>
+      </c>
+      <c r="F14" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14" s="44">
+        <v>2.0</v>
+      </c>
+      <c r="J14" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="K14" s="50"/>
+      <c r="L14" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="M14" s="50">
+        <v>4.0</v>
+      </c>
+      <c r="N14" s="50">
         <v>46.0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="50">
-        <v>7.5</v>
-      </c>
-      <c r="D9" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="E9" s="51">
-        <v>1.5</v>
-      </c>
-      <c r="F9" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="H9" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="I9" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="K9" s="48"/>
-      <c r="L9" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="M9" s="48">
-        <v>20.0</v>
-      </c>
-      <c r="N9" s="48">
-        <v>49.0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46" t="s">
-        <v>49</v>
-      </c>
-      <c r="M10" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="N10" s="51">
-        <v>49.0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="49" t="s">
+    <row r="15">
+      <c r="A15" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="G11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="K11" s="50"/>
-      <c r="L11" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="M11" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="N11" s="48">
+      <c r="B15" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="K15" s="47"/>
+      <c r="L15" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="M15" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="N15" s="47">
         <v>47.0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" s="45" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="46">
-        <v>7.5</v>
-      </c>
-      <c r="D12" s="51">
-        <v>3.5</v>
-      </c>
-      <c r="E12" s="51">
-        <v>1.5</v>
-      </c>
-      <c r="F12" s="51">
-        <v>30.0</v>
-      </c>
-      <c r="G12" s="51">
-        <v>1.5</v>
-      </c>
-      <c r="H12" s="51">
-        <v>1.5</v>
-      </c>
-      <c r="I12" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="K12" s="51"/>
-      <c r="L12" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="M12" s="51">
-        <v>45.0</v>
-      </c>
-      <c r="N12" s="51">
-        <v>46.0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="50">
-        <v>8.0</v>
-      </c>
-      <c r="D13" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="51">
-        <v>1.5</v>
-      </c>
-      <c r="F13" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" s="50">
-        <v>18.0</v>
-      </c>
-      <c r="J13" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="K13" s="48"/>
-      <c r="L13" s="48" t="s">
+    <row r="16">
+      <c r="A16" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J16" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="K16" s="50"/>
+      <c r="L16" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="M16" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="N16" s="50">
+        <v>48.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="M13" s="48">
-        <v>30.0</v>
-      </c>
-      <c r="N13" s="48">
-        <v>49.0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="45" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="E14" s="46">
-        <v>1.5</v>
-      </c>
-      <c r="F14" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="G14" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" s="46">
-        <v>2.0</v>
-      </c>
-      <c r="J14" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="K14" s="51"/>
-      <c r="L14" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="M14" s="51">
-        <v>4.0</v>
-      </c>
-      <c r="N14" s="51">
-        <v>46.0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="49" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="E15" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="G15" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="H15" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="J15" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="K15" s="48"/>
-      <c r="L15" s="48" t="s">
-        <v>51</v>
-      </c>
-      <c r="M15" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="N15" s="48">
-        <v>47.0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="G16" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="H16" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="K16" s="51"/>
-      <c r="L16" s="51" t="s">
-        <v>17</v>
-      </c>
-      <c r="M16" s="51" t="s">
-        <v>52</v>
-      </c>
-      <c r="N16" s="51">
-        <v>48.0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="49" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="50">
+      <c r="C17" s="49">
         <v>7.0</v>
       </c>
-      <c r="D17" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17" s="51">
-        <v>1.5</v>
-      </c>
-      <c r="F17" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="G17" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="H17" s="48" t="s">
-        <v>17</v>
+      <c r="D17" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="50">
+        <v>1.5</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="47" t="s">
+        <v>12</v>
       </c>
       <c r="I17" s="53">
         <v>15.0</v>
       </c>
-      <c r="J17" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="K17" s="48"/>
-      <c r="L17" s="48" t="s">
-        <v>17</v>
-      </c>
-      <c r="M17" s="48">
+      <c r="J17" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="K17" s="47"/>
+      <c r="L17" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="M17" s="47">
         <v>25.0</v>
       </c>
-      <c r="N17" s="48">
+      <c r="N17" s="47">
         <v>49.0</v>
       </c>
     </row>

</xml_diff>